<commit_message>
local: 更新观察池 2026-08-07 15:08
</commit_message>
<xml_diff>
--- a/mx_stocks_screener/观察池_累计.xlsx
+++ b/mx_stocks_screener/观察池_累计.xlsx
@@ -2103,7 +2103,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>跟踪中</t>
+          <t>已跟踪</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>2.02</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2121,10 +2121,14 @@
           <t>2.25</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>4.02</t>
+        </is>
+      </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>3.12</t>
+          <t>4.02</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
@@ -2137,10 +2141,26 @@
           <t>-1.56</t>
         </is>
       </c>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
-      <c r="AA15" t="inlineStr"/>
-      <c r="AB15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>震荡收涨</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>3.84</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>4.92</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>-1.73</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2225,7 +2245,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>跟踪中</t>
+          <t>已跟踪</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -2235,7 +2255,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>0.51</t>
+          <t>6.64</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -2243,7 +2263,11 @@
           <t>10.01</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>10.01</t>
+        </is>
+      </c>
       <c r="V16" t="inlineStr">
         <is>
           <t>10.01</t>
@@ -2259,10 +2283,26 @@
           <t>5.26</t>
         </is>
       </c>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
-      <c r="AA16" t="inlineStr"/>
-      <c r="AB16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>高开高走</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>16.06</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>16.06</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>11.05</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2339,7 +2379,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>跟踪中</t>
+          <t>已跟踪</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2357,10 +2397,14 @@
           <t>-0.06</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr"/>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>0.94</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
@@ -2373,7 +2417,11 @@
           <t>-3.69</t>
         </is>
       </c>
-      <c r="Y17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>震荡收涨</t>
+        </is>
+      </c>
       <c r="Z17" t="inlineStr"/>
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr"/>
@@ -2461,7 +2509,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>跟踪中</t>
+          <t>已跟踪</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -2471,7 +2519,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>0.97</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -2479,10 +2527,14 @@
           <t>3.45</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr"/>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>5.53</t>
+        </is>
+      </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>3.99</t>
+          <t>5.53</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
@@ -2495,10 +2547,26 @@
           <t>-1.01</t>
         </is>
       </c>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
-      <c r="AA18" t="inlineStr"/>
-      <c r="AB18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>高开高走</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>5.27</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>5.7</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>-1.25</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2583,7 +2651,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>跟踪中</t>
+          <t>已跟踪</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2593,7 +2661,7 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>6.31</t>
+          <t>-0.02</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -2601,15 +2669,19 @@
           <t>0.98</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>6.13</t>
+        </is>
+      </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>3.75</t>
+          <t>6.13</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>5.42</t>
+          <t>6.13</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
@@ -2617,10 +2689,26 @@
           <t>-2.33</t>
         </is>
       </c>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
-      <c r="AA19" t="inlineStr"/>
-      <c r="AB19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>震荡收涨</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>6.42</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>6.42</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>-2.07</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">

</xml_diff>